<commit_message>
data(isobutanol): regenerate opt_* workbooks with intended (non-derated) k_7/k_8
These five parameter-distribution workbooks are git-tracked (force-added
past the *.xlsx ignore rule). With scenario-level enzyme burden now
enforced at the load_simulate choke point and opt_* flipped to burden-ON,
the workbooks must store INTENDED k_7/k_8 (the A-referenced burden derates
them at simulate) rather than the pre-derated k_7_eff/k_8_eff they baked in
before. Regenerated by analyses/build_opt_scenario_workbooks.py; all five
opt_* pins reproduce unchanged and smoke_test_9-13 exit 0. Without this,
HEAD's stale workbooks would double-derate on a fresh checkout.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_opt_EtOH_titer.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_opt_EtOH_titer.xlsx
@@ -2707,7 +2707,7 @@
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0.9551252957512781</v>
+        <v>1.203</v>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
@@ -2715,13 +2715,13 @@
         </is>
       </c>
       <c r="G50" s="3" t="n">
-        <v>0.7641002366010226</v>
+        <v>0.9624000000000001</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>0.9551252957512781</v>
+        <v>1.203</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>1.146150354901534</v>
+        <v>1.4436</v>
       </c>
       <c r="J50" s="3" t="n"/>
       <c r="K50" s="3" t="inlineStr">
@@ -2932,7 +2932,7 @@
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.4676382370719059</v>
+        <v>0.589</v>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
@@ -2940,13 +2940,13 @@
         </is>
       </c>
       <c r="G55" s="3" t="n">
-        <v>0.3741105896575248</v>
+        <v>0.4712</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>0.4676382370719059</v>
+        <v>0.589</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>0.561165884486287</v>
+        <v>0.7068</v>
       </c>
       <c r="J55" s="3" t="n"/>
       <c r="K55" s="3" t="inlineStr">

</xml_diff>